<commit_message>
Event Expense July 15 2024 changes
</commit_message>
<xml_diff>
--- a/TestData/LV_T2279_TMTI0036293_ApproveEventExpenseFormAsSecondLevelApproverSet1.xlsx
+++ b/TestData/LV_T2279_TMTI0036293_ApproveEventExpenseFormAsSecondLevelApproverSet1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vkumar0427\source\repos\SF_Automation\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{289FA6B7-0365-4C68-B115-376903CC51FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA22978A-F220-4EA2-8B3F-9F6B131BC47F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,6 +21,7 @@
     <sheet name="Approver" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -537,17 +538,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>55</v>
       </c>
@@ -555,7 +556,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>36</v>
       </c>
@@ -563,7 +564,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -571,7 +572,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>36</v>
       </c>
@@ -579,7 +580,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>55</v>
       </c>
@@ -595,14 +596,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{780E0E82-BFFE-42FB-A31B-AC0D9C5DE596}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>52</v>
       </c>
@@ -615,14 +616,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D588DDF-4567-4D40-8446-D6AC9693F696}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>54</v>
       </c>
@@ -635,25 +636,25 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -704,7 +705,7 @@
       </c>
       <c r="Q1" s="1"/>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>27</v>
       </c>
@@ -760,7 +761,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>27</v>
       </c>
@@ -816,7 +817,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>27</v>
       </c>
@@ -872,7 +873,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -928,7 +929,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>27</v>
       </c>
@@ -993,13 +994,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>31</v>
       </c>
@@ -1007,7 +1008,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -1018,7 +1019,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>35</v>
       </c>
@@ -1029,7 +1030,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>35</v>
       </c>
@@ -1040,7 +1041,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>35</v>
       </c>
@@ -1051,7 +1052,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>34</v>
       </c>
@@ -1081,13 +1082,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="19.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="19.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>31</v>
       </c>
@@ -1095,7 +1096,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>33</v>
       </c>
@@ -1106,7 +1107,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>33</v>
       </c>
@@ -1117,7 +1118,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>47</v>
       </c>
@@ -1128,7 +1129,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>47</v>
       </c>
@@ -1139,7 +1140,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>47</v>
       </c>

</xml_diff>